<commit_message>
Actualizar catalogo con nuevas obras WebP, fichas tecnicas, foto de portada y obra a pedido
</commit_message>
<xml_diff>
--- a/images/obras/Detaller técnicos de obras.xlsx
+++ b/images/obras/Detaller técnicos de obras.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="67">
   <si>
     <t>Detalles técnicos de obras</t>
   </si>
@@ -94,7 +94,7 @@
     <t xml:space="preserve">110 x 90 cm </t>
   </si>
   <si>
-    <t>Sin título - formato horizontal</t>
+    <t>Formato alargado</t>
   </si>
   <si>
     <t>Acrílico sobre papel</t>
@@ -103,13 +103,13 @@
     <t xml:space="preserve">40 x 120 cm </t>
   </si>
   <si>
-    <t xml:space="preserve">Sin título - cálidos </t>
+    <t xml:space="preserve">Cálidos </t>
   </si>
   <si>
     <t xml:space="preserve">60 x 50 cm </t>
   </si>
   <si>
-    <t xml:space="preserve">Sin título - neutros </t>
+    <t>Abstracción neutra</t>
   </si>
   <si>
     <t>110 x 110 cm</t>
@@ -118,10 +118,13 @@
     <t xml:space="preserve">No Disponible </t>
   </si>
   <si>
-    <t>Sin título - neutros y dorados</t>
+    <t>Neutros y dorados</t>
   </si>
   <si>
     <t xml:space="preserve">80 x 130 cm </t>
+  </si>
+  <si>
+    <t>Neutros</t>
   </si>
   <si>
     <t>Serie Botánica</t>
@@ -179,6 +182,15 @@
   </si>
   <si>
     <t xml:space="preserve">120 x 170 cm </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mezquita Omeya </t>
+  </si>
+  <si>
+    <t>Acrílico sobre bastidor - políptico</t>
+  </si>
+  <si>
+    <t>90 x 240 m</t>
   </si>
   <si>
     <t>A la Sombra</t>
@@ -984,10 +996,10 @@
     <row r="12">
       <c r="A12" s="6"/>
       <c r="B12" s="7" t="s">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>11</v>
@@ -996,7 +1008,7 @@
         <v>33</v>
       </c>
       <c r="F12" s="9">
-        <v>2017.0</v>
+        <v>2026.0</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>34</v>
@@ -1025,7 +1037,7 @@
     <row r="13">
       <c r="A13" s="6"/>
       <c r="B13" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>39</v>
@@ -1034,10 +1046,10 @@
         <v>11</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="F13" s="9">
-        <v>2021.0</v>
+        <v>2017.0</v>
       </c>
       <c r="G13" s="9" t="s">
         <v>34</v>
@@ -1066,22 +1078,22 @@
     <row r="14">
       <c r="A14" s="6"/>
       <c r="B14" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F14" s="9">
-        <v>2022.0</v>
+        <v>2021.0</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -1107,19 +1119,19 @@
     <row r="15">
       <c r="A15" s="6"/>
       <c r="B15" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>45</v>
-      </c>
       <c r="F15" s="9">
-        <v>2023.0</v>
+        <v>2022.0</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>17</v>
@@ -1148,19 +1160,19 @@
     <row r="16">
       <c r="A16" s="6"/>
       <c r="B16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>48</v>
-      </c>
       <c r="F16" s="9">
-        <v>2017.0</v>
+        <v>2023.0</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>17</v>
@@ -1188,23 +1200,23 @@
     </row>
     <row r="17">
       <c r="A17" s="6"/>
-      <c r="B17" s="9" t="s">
-        <v>46</v>
+      <c r="B17" s="7" t="s">
+        <v>47</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F17" s="9">
-        <v>2025.0</v>
+        <v>2017.0</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -1230,16 +1242,16 @@
     <row r="18">
       <c r="A18" s="6"/>
       <c r="B18" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F18" s="9">
         <v>2025.0</v>
@@ -1271,22 +1283,22 @@
     <row r="19">
       <c r="A19" s="6"/>
       <c r="B19" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="F19" s="9">
-        <v>2024.0</v>
+        <v>2025.0</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1311,8 +1323,8 @@
     </row>
     <row r="20">
       <c r="A20" s="6"/>
-      <c r="B20" s="7" t="s">
-        <v>46</v>
+      <c r="B20" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>54</v>
@@ -1321,13 +1333,13 @@
         <v>11</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="F20" s="9">
-        <v>2020.0</v>
+        <v>2024.0</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -1353,22 +1365,22 @@
     <row r="21">
       <c r="A21" s="6"/>
       <c r="B21" s="7" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>11</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F21" s="9">
-        <v>2024.0</v>
+        <v>2020.0</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1394,22 +1406,22 @@
     <row r="22">
       <c r="A22" s="6"/>
       <c r="B22" s="7" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C22" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>11</v>
-      </c>
       <c r="E22" s="10" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="F22" s="9">
-        <v>2025.0</v>
+        <v>2018.0</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
@@ -1435,19 +1447,19 @@
     <row r="23">
       <c r="A23" s="6"/>
       <c r="B23" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F23" s="9">
-        <v>2025.0</v>
+        <v>2024.0</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>17</v>
@@ -1476,22 +1488,22 @@
     <row r="24">
       <c r="A24" s="6"/>
       <c r="B24" s="7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="F24" s="9">
-        <v>2023.0</v>
+        <v>2025.0</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
@@ -1516,8 +1528,24 @@
     </row>
     <row r="25">
       <c r="A25" s="6"/>
-      <c r="B25" s="9"/>
-      <c r="E25" s="11"/>
+      <c r="B25" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F25" s="9">
+        <v>2025.0</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>17</v>
+      </c>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -1541,8 +1569,24 @@
     </row>
     <row r="26">
       <c r="A26" s="6"/>
-      <c r="B26" s="9"/>
-      <c r="E26" s="11"/>
+      <c r="B26" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F26" s="9">
+        <v>2023.0</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
@@ -1565,14 +1609,9 @@
       <c r="AB26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
+      <c r="A27" s="6"/>
+      <c r="B27" s="9"/>
+      <c r="E27" s="11"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
@@ -1595,14 +1634,9 @@
       <c r="AB27" s="2"/>
     </row>
     <row r="28">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
+      <c r="A28" s="6"/>
+      <c r="B28" s="9"/>
+      <c r="E28" s="11"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
@@ -30934,12 +30968,72 @@
       <c r="AA1005" s="2"/>
       <c r="AB1005" s="2"/>
     </row>
+    <row r="1006">
+      <c r="A1006" s="2"/>
+      <c r="B1006" s="2"/>
+      <c r="C1006" s="2"/>
+      <c r="D1006" s="2"/>
+      <c r="E1006" s="3"/>
+      <c r="F1006" s="2"/>
+      <c r="G1006" s="2"/>
+      <c r="H1006" s="2"/>
+      <c r="I1006" s="2"/>
+      <c r="J1006" s="2"/>
+      <c r="K1006" s="2"/>
+      <c r="L1006" s="2"/>
+      <c r="M1006" s="2"/>
+      <c r="N1006" s="2"/>
+      <c r="O1006" s="2"/>
+      <c r="P1006" s="2"/>
+      <c r="Q1006" s="2"/>
+      <c r="R1006" s="2"/>
+      <c r="S1006" s="2"/>
+      <c r="T1006" s="2"/>
+      <c r="U1006" s="2"/>
+      <c r="V1006" s="2"/>
+      <c r="W1006" s="2"/>
+      <c r="X1006" s="2"/>
+      <c r="Y1006" s="2"/>
+      <c r="Z1006" s="2"/>
+      <c r="AA1006" s="2"/>
+      <c r="AB1006" s="2"/>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="2"/>
+      <c r="B1007" s="2"/>
+      <c r="C1007" s="2"/>
+      <c r="D1007" s="2"/>
+      <c r="E1007" s="3"/>
+      <c r="F1007" s="2"/>
+      <c r="G1007" s="2"/>
+      <c r="H1007" s="2"/>
+      <c r="I1007" s="2"/>
+      <c r="J1007" s="2"/>
+      <c r="K1007" s="2"/>
+      <c r="L1007" s="2"/>
+      <c r="M1007" s="2"/>
+      <c r="N1007" s="2"/>
+      <c r="O1007" s="2"/>
+      <c r="P1007" s="2"/>
+      <c r="Q1007" s="2"/>
+      <c r="R1007" s="2"/>
+      <c r="S1007" s="2"/>
+      <c r="T1007" s="2"/>
+      <c r="U1007" s="2"/>
+      <c r="V1007" s="2"/>
+      <c r="W1007" s="2"/>
+      <c r="X1007" s="2"/>
+      <c r="Y1007" s="2"/>
+      <c r="Z1007" s="2"/>
+      <c r="AA1007" s="2"/>
+      <c r="AB1007" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G3:G24">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="G3:G26">
       <formula1>"No Disponible ,Disponible "</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>